<commit_message>
Align Companies workbook v2 with live module
</commit_message>
<xml_diff>
--- a/temp/WRCF End-to-End Test Cases_reverified-v2.xlsx
+++ b/temp/WRCF End-to-End Test Cases_reverified-v2.xlsx
@@ -9160,7 +9160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W22"/>
+  <dimension ref="A1:W60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11.5703125" customWidth="1" min="1" max="1"/>
@@ -9306,7 +9306,7 @@
     <row r="2" ht="60" customHeight="1">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-001</t>
+          <t>COMP-CUR-001</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -9316,37 +9316,37 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Company dashboard load</t>
+          <t>Manage Company load</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>Verify company WRCF dashboard loads using the referenced industry template</t>
+          <t>Manage Company loads with list and selected company details</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>Authorized Company Admin logged in; company references an industry template</t>
+          <t>Authorized user logged in; at least one company exists</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>Company tenant linked to industry template</t>
+          <t>Existing company record</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>1. Open Company WRCF dashboard for a company tenant</t>
+          <t>1. Open Manage Company</t>
         </is>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>Company dashboard loads in the context of the referenced industry template</t>
+          <t>Manage Company page loads, list is visible, and selected company details are shown</t>
         </is>
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Functional / UI</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr">
@@ -9356,27 +9356,27 @@
       </c>
       <c r="K2" s="8" t="inlineStr">
         <is>
-          <t>Company references Industry template</t>
+          <t>Live Manage Company CRUD baseline</t>
         </is>
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>Company Dashboard</t>
+          <t>Manage Company screen</t>
         </is>
       </c>
       <c r="M2" s="9" t="inlineStr">
         <is>
-          <t>tenants.type='COMPANY' with linked industry/source context</t>
+          <t>List/detail layout</t>
         </is>
       </c>
       <c r="N2" s="8" t="inlineStr">
         <is>
-          <t>Company tenant</t>
+          <t>Login/Auth module</t>
         </is>
       </c>
       <c r="O2" s="14" t="inlineStr">
         <is>
-          <t>@future</t>
+          <t>@stable</t>
         </is>
       </c>
       <c r="P2" s="18" t="inlineStr">
@@ -9391,34 +9391,29 @@
       </c>
       <c r="R2" s="11" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="S2" s="11" t="inlineStr">
         <is>
-          <t>product-gap</t>
+          <t>none</t>
         </is>
       </c>
       <c r="T2" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live UI at /manage-company is a CRUD management page and does not expose the company WRCF dashboard/template-linked landing surface described in the wor</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>failed: company WRCF dashboard surface missing</t>
+          <t>Verified passing in the 11:11 PM @ 03/04/26 rerun.</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>failed: Current live UI at /manage-company is a CRUD management page and does not expose the compa</t>
+          <t>passed</t>
         </is>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-002</t>
+          <t>COMP-CUR-002</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -9428,32 +9423,32 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Version summary</t>
+          <t>Company search</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>Verify dashboard shows Industry Version, Company Version, and Overrides count</t>
+          <t>Search filters the company list</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>Company WRCF exists</t>
+          <t>Manage Company loaded with at least one company</t>
         </is>
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Industry v4.2, Company v4.2-C1, Overrides=27</t>
+          <t>Search term and unmatched term</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>1. Open Company Dashboard 2. Observe version summary area</t>
+          <t>1. Enter unmatched search 2. Clear search</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>Dashboard shows Industry Version, Company Version, and Overrides count</t>
+          <t>List shows no-result state for unmatched term and restores the list when cleared</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
@@ -9463,37 +9458,37 @@
       </c>
       <c r="J3" s="8" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K3" s="8" t="inlineStr">
         <is>
-          <t>Company dashboard shows Industry Version, Company Version, Overrides</t>
+          <t>Live Manage Company CRUD baseline</t>
         </is>
       </c>
       <c r="L3" s="8" t="inlineStr">
         <is>
-          <t>Company Dashboard</t>
+          <t>Manage Company screen</t>
         </is>
       </c>
       <c r="M3" s="9" t="inlineStr">
         <is>
-          <t>wrcf_versions + company delta metadata</t>
+          <t>Search behavior</t>
         </is>
       </c>
       <c r="N3" s="8" t="inlineStr">
         <is>
-          <t>Company tenant + versions</t>
+          <t>Company list data</t>
         </is>
       </c>
       <c r="O3" s="14" t="inlineStr">
         <is>
-          <t>@future</t>
+          <t>@stable</t>
         </is>
       </c>
       <c r="P3" s="18" t="inlineStr">
         <is>
-          <t>@p0</t>
+          <t>@p1</t>
         </is>
       </c>
       <c r="Q3" s="22" t="inlineStr">
@@ -9503,34 +9498,29 @@
       </c>
       <c r="R3" s="11" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="S3" s="11" t="inlineStr">
         <is>
-          <t>product-gap</t>
+          <t>none</t>
         </is>
       </c>
       <c r="T3" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose a company-WRCF version summary area with Industry Version, Company Version, or Overrides count.</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>failed: version summary surface missing</t>
+          <t>Verified passing in the 11:11 PM @ 03/04/26 rerun.</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t xml:space="preserve">failed: Current live Manage Company page does not expose a company-WRCF version summary area with </t>
+          <t>passed</t>
         </is>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-003</t>
+          <t>COMP-CUR-003</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -9540,72 +9530,72 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Dashboard sections</t>
+          <t>Create validation</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Verify dashboard shows Structural Overrides, Capability Overrides, Role Overrides, and Upgrade Available sections when applicable</t>
+          <t>Create form blocks save when Name is empty</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Company dashboard loaded</t>
+          <t>Manage Company loaded</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>Company with overrides and/or upgrade state</t>
+          <t>Blank name</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>1. Open Company Dashboard 2. Observe visible sections</t>
+          <t>1. Click Add 2. Click Save</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>Dashboard shows Structural Overrides, Capability Overrides, Role Overrides, and Upgrade Available when applicable</t>
+          <t>Validation shows Name is required</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>Functional / UI</t>
+          <t>Functional / Validation</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="K4" s="8" t="inlineStr">
         <is>
-          <t>Company dashboard sections defined in company WRCF flow</t>
+          <t>Live Manage Company CRUD baseline</t>
         </is>
       </c>
       <c r="L4" s="8" t="inlineStr">
         <is>
-          <t>Company Dashboard</t>
+          <t>Manage Company form</t>
         </is>
       </c>
       <c r="M4" s="9" t="inlineStr">
         <is>
-          <t>Override categories / upgrade state</t>
+          <t>Required-name validation</t>
         </is>
       </c>
       <c r="N4" s="8" t="inlineStr">
         <is>
-          <t>Company tenant</t>
+          <t>Create company form</t>
         </is>
       </c>
       <c r="O4" s="14" t="inlineStr">
         <is>
-          <t>@future</t>
+          <t>@stable</t>
         </is>
       </c>
       <c r="P4" s="18" t="inlineStr">
         <is>
-          <t>@p1</t>
+          <t>@p0</t>
         </is>
       </c>
       <c r="Q4" s="22" t="inlineStr">
@@ -9615,34 +9605,29 @@
       </c>
       <c r="R4" s="11" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="S4" s="11" t="inlineStr">
         <is>
-          <t>product-gap</t>
+          <t>none</t>
         </is>
       </c>
       <c r="T4" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose company-WRCF override sections or upgrade state sections.</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>failed: override and upgrade sections missing</t>
+          <t>Verified passing in the 11:11 PM @ 03/04/26 rerun.</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>failed: Current live Manage Company page does not expose company-WRCF override sections or upgrade</t>
+          <t>passed</t>
         </is>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-004</t>
+          <t>COMP-CUR-004</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -9652,72 +9637,72 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Company Admin permissions</t>
+          <t>Edit prefill</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Verify Company Admin can perform override actions only</t>
+          <t>Edit form opens with selected company prefilled</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Company Admin user exists</t>
+          <t>Manage Company loaded with selected company</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Company Admin account</t>
+          <t>Existing selected company</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>1. Login as Company Admin 2. Open company WRCF</t>
+          <t>1. Click Edit</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>User can perform override actions but cannot perform industry-master full-edit actions</t>
+          <t>Edit form opens with selected company values prefilled</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>Role-based / Security</t>
+          <t>Functional / UI</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K5" s="8" t="inlineStr">
         <is>
-          <t>Company Admin: Override only</t>
+          <t>Live Manage Company CRUD baseline</t>
         </is>
       </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
-          <t>Company Dashboard / Company Role Adjustments</t>
+          <t>Manage Company form</t>
         </is>
       </c>
       <c r="M5" s="9" t="inlineStr">
         <is>
-          <t>Permissions layer</t>
+          <t>Edit prefill</t>
         </is>
       </c>
       <c r="N5" s="8" t="inlineStr">
         <is>
-          <t>RBAC</t>
+          <t>Selected company detail</t>
         </is>
       </c>
       <c r="O5" s="14" t="inlineStr">
         <is>
-          <t>@future</t>
+          <t>@stable</t>
         </is>
       </c>
       <c r="P5" s="18" t="inlineStr">
         <is>
-          <t>@p0</t>
+          <t>@p1</t>
         </is>
       </c>
       <c r="Q5" s="22" t="inlineStr">
@@ -9727,34 +9712,29 @@
       </c>
       <c r="R5" s="11" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="S5" s="11" t="inlineStr">
         <is>
-          <t>runtime/data</t>
+          <t>none</t>
         </is>
       </c>
       <c r="T5" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: This workbook permission case depends on a company-WRCF override surface and a dedicated Company Admin account matrix that are not represented in the current li</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Verified passing in the 11:11 PM @ 03/04/26 rerun.</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>failed: This workbook permission case depends on a company-WRCF override surface and a dedicated C</t>
+          <t>passed</t>
         </is>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-005</t>
+          <t>COMP-CUR-005</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -9764,72 +9744,72 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Industry Architect permissions</t>
+          <t>Preview flow</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Verify Industry Architect has full edit access to master WRCF flows</t>
+          <t>Preview opens from edit and returns back to list/detail view</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Industry Architect user exists</t>
+          <t>Edit form available for selected company</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>Industry Architect account</t>
+          <t>Existing selected company</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>1. Login as Industry Architect 2. Open relevant WRCF context</t>
+          <t>1. Click Edit 2. Click Preview 3. Click Back</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Industry Architect has full edit access to master WRCF flows</t>
+          <t>Preview opens and Back returns to list/detail view</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>Role-based / Security</t>
+          <t>Functional / UI</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr">
         <is>
-          <t>Industry Architect: Full edit access</t>
+          <t>Live Manage Company CRUD baseline</t>
         </is>
       </c>
       <c r="L6" s="8" t="inlineStr">
         <is>
-          <t>Industry / Company WRCF views</t>
+          <t>Manage Company preview</t>
         </is>
       </c>
       <c r="M6" s="9" t="inlineStr">
         <is>
-          <t>Permissions layer</t>
+          <t>Preview/back flow</t>
         </is>
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
-          <t>RBAC</t>
+          <t>Edit form</t>
         </is>
       </c>
       <c r="O6" s="14" t="inlineStr">
         <is>
-          <t>@future</t>
+          <t>@stable</t>
         </is>
       </c>
       <c r="P6" s="18" t="inlineStr">
         <is>
-          <t>@p2</t>
+          <t>@p1</t>
         </is>
       </c>
       <c r="Q6" s="22" t="inlineStr">
@@ -9839,34 +9819,29 @@
       </c>
       <c r="R6" s="11" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="S6" s="11" t="inlineStr">
         <is>
-          <t>runtime/data</t>
+          <t>none</t>
         </is>
       </c>
       <c r="T6" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: This workbook permission case targets industry-master WRCF flows rather than the current Manage Company CRUD page and needs dedicated RBAC accounts to verify.</t>
-        </is>
-      </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Verified passing in the 11:11 PM @ 03/04/26 rerun.</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>failed: This workbook permission case targets industry-master WRCF flows rather than the current M</t>
+          <t>passed</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-006</t>
+          <t>COMP-CUR-006</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -9876,72 +9851,72 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Auditor permissions</t>
+          <t>Email validation</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Verify Auditor can only view and export company WRCF</t>
+          <t>Contact email format is validated before save</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Auditor user exists</t>
+          <t>Edit form open</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Auditor account</t>
+          <t>Invalid email</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>1. Login as Auditor 2. Open company WRCF</t>
+          <t>1. Open Edit 2. Enter invalid email 3. Click Save</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>Company data is viewable/exportable only; override actions are hidden or disabled</t>
+          <t>Validation shows Enter a valid email</t>
         </is>
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>Role-based / Security</t>
+          <t>Functional / Validation</t>
         </is>
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K7" s="8" t="inlineStr">
         <is>
-          <t>Auditor: View + export only</t>
+          <t>Live Manage Company CRUD baseline</t>
         </is>
       </c>
       <c r="L7" s="8" t="inlineStr">
         <is>
-          <t>Company Dashboard</t>
+          <t>Manage Company form</t>
         </is>
       </c>
       <c r="M7" s="9" t="inlineStr">
         <is>
-          <t>Permissions layer</t>
+          <t>Email format validation</t>
         </is>
       </c>
       <c r="N7" s="8" t="inlineStr">
         <is>
-          <t>RBAC</t>
+          <t>Edit form</t>
         </is>
       </c>
       <c r="O7" s="14" t="inlineStr">
         <is>
-          <t>@future</t>
+          <t>@stable</t>
         </is>
       </c>
       <c r="P7" s="18" t="inlineStr">
         <is>
-          <t>@p0</t>
+          <t>@p1</t>
         </is>
       </c>
       <c r="Q7" s="22" t="inlineStr">
@@ -9951,34 +9926,29 @@
       </c>
       <c r="R7" s="11" t="inlineStr">
         <is>
-          <t>fail</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="S7" s="11" t="inlineStr">
         <is>
-          <t>product-gap</t>
+          <t>none</t>
         </is>
       </c>
       <c r="T7" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the company-WRCF export surface and this role-based case needs a dedicated Auditor account.</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Verified passing in the 11:11 PM @ 03/04/26 rerun.</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t xml:space="preserve">failed: Current live Manage Company page does not expose the company-WRCF export surface and this </t>
+          <t>passed</t>
         </is>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-007</t>
+          <t>COMP-E2E-001</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -9988,62 +9958,62 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Employee permissions</t>
+          <t>Company dashboard load</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Verify Employee can only view role capability requirements</t>
+          <t>Verify company WRCF dashboard loads using the referenced industry template</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Employee user exists</t>
+          <t>Authorized Company Admin logged in; company references an industry template</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Employee account</t>
+          <t>Company tenant linked to industry template</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>1. Login as Employee 2. Open company role requirement view</t>
+          <t>1. Open Company WRCF dashboard for a company tenant</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Employee can view role capability requirements only and cannot access override actions</t>
+          <t>Company dashboard loads in the context of the referenced industry template</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Role-based / Security</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
-          <t>Employee: View role capability requirements only</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>Company role requirement view</t>
+          <t>Company WRCF dashboard</t>
         </is>
       </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
-          <t>Permissions layer</t>
+          <t>Template-linked company WRCF load</t>
         </is>
       </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
-          <t>RBAC</t>
+          <t>Industry template linkage</t>
         </is>
       </c>
       <c r="O8" s="14" t="inlineStr">
@@ -10053,7 +10023,7 @@
       </c>
       <c r="P8" s="18" t="inlineStr">
         <is>
-          <t>@p1</t>
+          <t>@p0</t>
         </is>
       </c>
       <c r="Q8" s="22" t="inlineStr">
@@ -10073,24 +10043,19 @@
       </c>
       <c r="T8" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live runtime does not expose the company role requirement view described in the workbook and this case needs an Employee account.</t>
-        </is>
-      </c>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live UI at /manage-company is a CRUD management page and does not expose the company WRCF dashboard/template-linked landing surface described in the workbook.</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>failed: Current live runtime does not expose the company role requirement view described in the wo</t>
+          <t>failed: Current live UI at /manage-company is a CRUD management page and does not expose the compa</t>
         </is>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-008</t>
+          <t>COMP-E2E-002</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -10100,37 +10065,37 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Customize capability instance</t>
+          <t>Version summary</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>Verify company can save company-specific capability-instance overrides without duplicating full master data</t>
+          <t>Verify dashboard shows Industry Version, Company Version, and Overrides count</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Company Admin logged in; base industry CI exists</t>
+          <t>Company WRCF exists</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Master CI plus company override for selected fields</t>
+          <t>Industry v4.2, Company v4.2-C1, Overrides=27</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>1. Open company capability-instance customization 2. Change allowed override fields 3. Save</t>
+          <t>1. Open Company Dashboard 2. Observe version summary area</t>
         </is>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>System stores only the company-specific override fields and uses master + override model</t>
+          <t>Dashboard shows Industry Version, Company Version, and Overrides count</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>Functional / Data integrity</t>
+          <t>Functional / UI</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
@@ -10140,22 +10105,22 @@
       </c>
       <c r="K9" s="8" t="inlineStr">
         <is>
-          <t>Only store company-specific overrides; no duplication explosion</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L9" s="8" t="inlineStr">
         <is>
-          <t>Customize Capability Instance</t>
+          <t>Company WRCF dashboard</t>
         </is>
       </c>
       <c r="M9" s="9" t="inlineStr">
         <is>
-          <t>Hybrid delta model / override layer</t>
+          <t>Version summary</t>
         </is>
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>Company tenant + source template CI</t>
+          <t>Company WRCF exists</t>
         </is>
       </c>
       <c r="O9" s="14" t="inlineStr">
@@ -10185,24 +10150,19 @@
       </c>
       <c r="T9" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose company-specific capability-instance override editing or the hybrid master-plus-override save flow.</t>
-        </is>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose a company-WRCF version summary area with Industry Version, Company Version, or Overrides count.</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>failed: Current live Manage Company page does not expose company-specific capability-instance over</t>
+          <t xml:space="preserve">failed: Current live Manage Company page does not expose a company-WRCF version summary area with </t>
         </is>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-009</t>
+          <t>COMP-E2E-003</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -10212,62 +10172,62 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Runtime merge view</t>
+          <t>Dashboard sections</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Verify runtime view overlays company overrides on top of the industry master</t>
+          <t>Verify dashboard shows Structural Overrides, Capability Overrides, Role Overrides, and Upgrade Available sections when applicable</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>Master template and company override exist</t>
+          <t>Company dashboard loaded</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Master field + overridden field</t>
+          <t>Company with overrides and/or upgrade state</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>1. Load final company WRCF view for overridden context</t>
+          <t>1. Open Company Dashboard 2. Observe visible sections</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>System renders master values together with company override values in the final view</t>
+          <t>Dashboard shows Structural Overrides, Capability Overrides, Role Overrides, and Upgrade Available when applicable</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>Functional / Data integrity</t>
+          <t>Functional / UI</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K10" s="8" t="inlineStr">
         <is>
-          <t>At runtime, system loads master then overlays company overrides</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L10" s="8" t="inlineStr">
         <is>
-          <t>Company Dashboard / final rendered view</t>
+          <t>Company WRCF dashboard</t>
         </is>
       </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>Hybrid delta model runtime merge</t>
+          <t>Override sections</t>
         </is>
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
-          <t>Company tenant + source template</t>
+          <t>Dashboard loaded</t>
         </is>
       </c>
       <c r="O10" s="14" t="inlineStr">
@@ -10277,7 +10237,7 @@
       </c>
       <c r="P10" s="18" t="inlineStr">
         <is>
-          <t>@p0</t>
+          <t>@p1</t>
         </is>
       </c>
       <c r="Q10" s="22" t="inlineStr">
@@ -10297,24 +10257,19 @@
       </c>
       <c r="T10" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the final merged company-WRCF runtime view described in the workbook.</t>
-        </is>
-      </c>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose company-WRCF override sections or upgrade state sections.</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>failed: Current live Manage Company page does not expose the final merged company-WRCF runtime vie</t>
+          <t>failed: Current live Manage Company page does not expose company-WRCF override sections or upgrade</t>
         </is>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-010</t>
+          <t>COMP-E2E-004</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -10324,62 +10279,62 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Role variant comparison</t>
+          <t>Company Admin permissions</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Verify company role adjustments show Industry Role Template and Company Role Variant</t>
+          <t>Verify Company Admin can perform override actions only</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>Company has industry role template and one company role variant</t>
+          <t>Company Admin user exists</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Base role plus company variant</t>
+          <t>Company Admin account</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>1. Open Company Role Adjustments</t>
+          <t>1. Login as Company Admin 2. Open company WRCF</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>System shows Industry Role Template and Company Role Variant comparison</t>
+          <t>User can perform override actions but cannot perform industry-master full-edit actions</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>Functional / UI</t>
+          <t>Role-based / Security</t>
         </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="K11" s="8" t="inlineStr">
         <is>
-          <t>UI shows Industry Role Template and Company Role Variant</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L11" s="8" t="inlineStr">
         <is>
-          <t>Company Role Adjustments</t>
+          <t>Company WRCF RBAC</t>
         </is>
       </c>
       <c r="M11" s="9" t="inlineStr">
         <is>
-          <t>Role override comparison view</t>
+          <t>Company Admin permissions</t>
         </is>
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>Industry role + company variant</t>
+          <t>Company Admin account</t>
         </is>
       </c>
       <c r="O11" s="14" t="inlineStr">
@@ -10389,7 +10344,7 @@
       </c>
       <c r="P11" s="18" t="inlineStr">
         <is>
-          <t>@p1</t>
+          <t>@p0</t>
         </is>
       </c>
       <c r="Q11" s="22" t="inlineStr">
@@ -10404,29 +10359,24 @@
       </c>
       <c r="S11" s="11" t="inlineStr">
         <is>
-          <t>product-gap</t>
+          <t>runtime/data</t>
         </is>
       </c>
       <c r="T11" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose Company Role Adjustments or Industry Role Template vs Company Role Variant comparison.</t>
-        </is>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: This workbook permission case depends on a company-WRCF override surface and a dedicated Company Admin account matrix that are not represented in the current live Manage Company page/runtime.</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>failed: Current live Manage Company page does not expose Company Role Adjustments or Industry Role</t>
+          <t>failed: This workbook permission case depends on a company-WRCF override surface and a dedicated C</t>
         </is>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-011</t>
+          <t>COMP-E2E-005</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -10436,62 +10386,62 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Role variant color coding</t>
+          <t>Industry Architect permissions</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Verify comparison uses color coding for same, overridden, and removed items</t>
+          <t>Verify Industry Architect has full edit access to master WRCF flows</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Comparison screen open</t>
+          <t>Industry Architect user exists</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Mixed same/overridden/removed items</t>
+          <t>Industry Architect account</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>1. Open role comparison screen 2. Observe status colors</t>
+          <t>1. Login as Industry Architect 2. Open relevant WRCF context</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>Green marks same as industry, Orange marks overridden, and Red marks removed</t>
+          <t>Industry Architect has full edit access to master WRCF flows</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>UI / Requirement validation</t>
+          <t>Role-based / Security</t>
         </is>
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr">
         <is>
-          <t>Color coding: Green same, Orange overridden, Red removed</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L12" s="8" t="inlineStr">
         <is>
-          <t>Company Role Adjustments</t>
+          <t>WRCF RBAC</t>
         </is>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>Comparison-state rendering</t>
+          <t>Industry Architect permissions</t>
         </is>
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>Industry role + company variant</t>
+          <t>Industry Architect account</t>
         </is>
       </c>
       <c r="O12" s="14" t="inlineStr">
@@ -10516,29 +10466,24 @@
       </c>
       <c r="S12" s="11" t="inlineStr">
         <is>
-          <t>product-gap</t>
+          <t>runtime/data</t>
         </is>
       </c>
       <c r="T12" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the workbook role-comparison screen needed for this color-coding validation.</t>
-        </is>
-      </c>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: This workbook permission case targets industry-master WRCF flows rather than the current Manage Company CRUD page and needs dedicated RBAC accounts to verify.</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>failed: Current live Manage Company page does not expose the workbook role-comparison screen neede</t>
+          <t>failed: This workbook permission case targets industry-master WRCF flows rather than the current M</t>
         </is>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-012</t>
+          <t>COMP-E2E-006</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -10548,62 +10493,62 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Add internal company role</t>
+          <t>Auditor permissions</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Verify company can add a new internal role</t>
+          <t>Verify Auditor can only view and export company WRCF</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Company Admin logged in</t>
+          <t>Auditor user exists</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>Unique internal role name</t>
+          <t>Auditor account</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>1. Open Company Role Adjustments 2. Add new internal role 3. Save</t>
+          <t>1. Login as Auditor 2. Open company WRCF</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>New internal company role is added to the company variant</t>
+          <t>Company data is viewable/exportable only; override actions are hidden or disabled</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Role-based / Security</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="K13" s="8" t="inlineStr">
         <is>
-          <t>Company can add new internal roles</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L13" s="8" t="inlineStr">
         <is>
-          <t>Company Role Adjustments</t>
+          <t>Company WRCF RBAC</t>
         </is>
       </c>
       <c r="M13" s="9" t="inlineStr">
         <is>
-          <t>Company role override layer</t>
+          <t>Auditor permissions</t>
         </is>
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>Company tenant</t>
+          <t>Auditor account</t>
         </is>
       </c>
       <c r="O13" s="14" t="inlineStr">
@@ -10613,7 +10558,7 @@
       </c>
       <c r="P13" s="18" t="inlineStr">
         <is>
-          <t>@p1</t>
+          <t>@p0</t>
         </is>
       </c>
       <c r="Q13" s="22" t="inlineStr">
@@ -10633,24 +10578,19 @@
       </c>
       <c r="T13" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the company role-variant creation surface described in the workbook.</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the company-WRCF export surface and this role-based case needs a dedicated Auditor account.</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>failed: Current live Manage Company page does not expose the company role-variant creation surface</t>
+          <t xml:space="preserve">failed: Current live Manage Company page does not expose the company-WRCF export surface and this </t>
         </is>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-013</t>
+          <t>COMP-E2E-007</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -10660,37 +10600,37 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Adjust capability weight</t>
+          <t>Employee permissions</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Verify company can adjust capability weights in the company role variant</t>
+          <t>Verify Employee can only view role capability requirements</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Company role variant exists</t>
+          <t>Employee user exists</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Changed weight for one mapped CI</t>
+          <t>Employee account</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>1. Open a company role variant 2. Adjust capability weight 3. Save</t>
+          <t>1. Login as Employee 2. Open company role requirement view</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>Updated capability weight is saved in the company role variant</t>
+          <t>Employee can view role capability requirements only and cannot access override actions</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Role-based / Security</t>
         </is>
       </c>
       <c r="J14" s="8" t="inlineStr">
@@ -10700,22 +10640,22 @@
       </c>
       <c r="K14" s="8" t="inlineStr">
         <is>
-          <t>Company can adjust capability weights</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L14" s="8" t="inlineStr">
         <is>
-          <t>Company Role Adjustments</t>
+          <t>Company WRCF RBAC</t>
         </is>
       </c>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Company override on role mapping weight</t>
+          <t>Employee permissions</t>
         </is>
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>Company role variant</t>
+          <t>Employee account</t>
         </is>
       </c>
       <c r="O14" s="14" t="inlineStr">
@@ -10745,24 +10685,19 @@
       </c>
       <c r="T14" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose company role-variant capability weight adjustment.</t>
-        </is>
-      </c>
-      <c r="V14" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live runtime does not expose the company role requirement view described in the workbook and this case needs an Employee account.</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>failed: Current live Manage Company page does not expose company role-variant capability weight ad</t>
+          <t>failed: Current live runtime does not expose the company role requirement view described in the wo</t>
         </is>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-014</t>
+          <t>COMP-E2E-008</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -10772,62 +10707,62 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Change certification threshold</t>
+          <t>Customize capability instance</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Verify company can change certification threshold in the company role variant</t>
+          <t>Verify company can save company-specific capability-instance overrides without duplicating full master data</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>Company role variant exists</t>
+          <t>Company Admin logged in; base industry CI exists</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>New threshold value</t>
+          <t>Master CI plus company override for selected fields</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>1. Open company role variant 2. Change certification threshold 3. Save</t>
+          <t>1. Open company capability-instance customization 2. Change allowed override fields 3. Save</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>Updated certification threshold is saved in the company role variant</t>
+          <t>System stores only the company-specific override fields and uses master + override model</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
-          <t>Functional</t>
+          <t>Functional / Data integrity</t>
         </is>
       </c>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="K15" s="8" t="inlineStr">
         <is>
-          <t>Company can change certification threshold</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L15" s="8" t="inlineStr">
         <is>
-          <t>Company Role Adjustments</t>
+          <t>Company capability override</t>
         </is>
       </c>
       <c r="M15" s="9" t="inlineStr">
         <is>
-          <t>Company role variant threshold override</t>
+          <t>Override save model</t>
         </is>
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>Company role variant</t>
+          <t>Base industry CI exists</t>
         </is>
       </c>
       <c r="O15" s="14" t="inlineStr">
@@ -10837,7 +10772,7 @@
       </c>
       <c r="P15" s="18" t="inlineStr">
         <is>
-          <t>@p1</t>
+          <t>@p0</t>
         </is>
       </c>
       <c r="Q15" s="22" t="inlineStr">
@@ -10857,24 +10792,19 @@
       </c>
       <c r="T15" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose company role-variant certification-threshold override editing.</t>
-        </is>
-      </c>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose company-specific capability-instance override editing or the hybrid master-plus-override save flow.</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>failed: Current live Manage Company page does not expose company role-variant certification-thresh</t>
+          <t>failed: Current live Manage Company page does not expose company-specific capability-instance over</t>
         </is>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-015</t>
+          <t>COMP-E2E-009</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -10884,37 +10814,37 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Upgrade available indicator</t>
+          <t>Runtime merge view</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Verify company sees Upgrade Available when industry publishes a newer version</t>
+          <t>Verify runtime view overlays company overrides on top of the industry master</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>Company references industry version 4.2; industry publishes 5.0</t>
+          <t>Master template and company override exist</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>Newer published industry version available</t>
+          <t>Master field + overridden field</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>1. Publish newer industry version 2. Open company dashboard</t>
+          <t>1. Load final company WRCF view for overridden context</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>Dashboard shows Upgrade Available with the newer industry version</t>
+          <t>System renders master values together with company override values in the final view</t>
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
-          <t>Functional / Versioning</t>
+          <t>Functional / Data integrity</t>
         </is>
       </c>
       <c r="J16" s="8" t="inlineStr">
@@ -10924,22 +10854,22 @@
       </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>When Industry updates, companies get Upgrade Available</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L16" s="8" t="inlineStr">
         <is>
-          <t>Company Dashboard</t>
+          <t>Company merged runtime view</t>
         </is>
       </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Industry/company version comparison</t>
+          <t>Master + override overlay</t>
         </is>
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>Industry version + company version</t>
+          <t>Master and company override</t>
         </is>
       </c>
       <c r="O16" s="14" t="inlineStr">
@@ -10969,24 +10899,19 @@
       </c>
       <c r="T16" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose industry/company WRCF version comparison or Upgrade Available state.</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the final merged company-WRCF runtime view described in the workbook.</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t xml:space="preserve">failed: Current live Manage Company page does not expose industry/company WRCF version comparison </t>
+          <t>failed: Current live Manage Company page does not expose the final merged company-WRCF runtime vie</t>
         </is>
       </c>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-016</t>
+          <t>COMP-E2E-010</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -10996,62 +10921,62 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Upgrade diff screen</t>
+          <t>Role variant comparison</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Verify upgrade flow shows diffs before applying update</t>
+          <t>Verify company role adjustments show Industry Role Template and Company Role Variant</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Upgrade available state exists</t>
+          <t>Company has industry role template and one company role variant</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>Changes include new CI / modified escalation / updated regulatory refs</t>
+          <t>Base role plus company variant</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>1. Open Upgrade Available 2. Review diff screen</t>
+          <t>1. Open Company Role Adjustments</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>System shows differences such as new capability instances, modified escalation levels, and updated regulatory references</t>
+          <t>System shows Industry Role Template and Company Role Variant comparison</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>Functional / Versioning</t>
+          <t>Functional / UI</t>
         </is>
       </c>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K17" s="8" t="inlineStr">
         <is>
-          <t>Upgrade &amp; Merge Flow shows diff before decision</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L17" s="8" t="inlineStr">
         <is>
-          <t>Upgrade &amp; Merge Flow</t>
+          <t>Company role adjustments</t>
         </is>
       </c>
       <c r="M17" s="9" t="inlineStr">
         <is>
-          <t>Diff against source template version</t>
+          <t>Role template vs variant</t>
         </is>
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>Industry version delta</t>
+          <t>Company role variant exists</t>
         </is>
       </c>
       <c r="O17" s="14" t="inlineStr">
@@ -11061,7 +10986,7 @@
       </c>
       <c r="P17" s="18" t="inlineStr">
         <is>
-          <t>@p0</t>
+          <t>@p1</t>
         </is>
       </c>
       <c r="Q17" s="22" t="inlineStr">
@@ -11081,24 +11006,19 @@
       </c>
       <c r="T17" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the workbook Upgrade &amp; Merge diff flow.</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose Company Role Adjustments or Industry Role Template vs Company Role Variant comparison.</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>failed: Current live Manage Company page does not expose the workbook Upgrade &amp; Merge diff flow.</t>
+          <t>failed: Current live Manage Company page does not expose Company Role Adjustments or Industry Role</t>
         </is>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-017</t>
+          <t>COMP-E2E-011</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -11108,62 +11028,62 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Accept all upgrade</t>
+          <t>Role variant color coding</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Verify Accept All applies all industry updates and generates the next company version</t>
+          <t>Verify comparison uses color coding for same, overridden, and removed items</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>Upgrade available state exists</t>
+          <t>Comparison screen open</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Company on 4.2-C1; industry on 5.0</t>
+          <t>Mixed same/overridden/removed items</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>1. Open upgrade flow 2. Click Accept All 3. Confirm</t>
+          <t>1. Open role comparison screen 2. Observe status colors</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>All applicable updates are applied and a new company version is generated</t>
+          <t>Green marks same as industry, Orange marks overridden, and Red marks removed</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>Functional / Versioning</t>
+          <t>UI / Requirement validation</t>
         </is>
       </c>
       <c r="J18" s="8" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K18" s="8" t="inlineStr">
         <is>
-          <t>Final step generates next company version after accepted updates</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L18" s="8" t="inlineStr">
         <is>
-          <t>Upgrade &amp; Merge Flow</t>
+          <t>Company role comparison</t>
         </is>
       </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Company version generation after merge</t>
+          <t>Color coding</t>
         </is>
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>Industry version delta + company version</t>
+          <t>Comparison screen open</t>
         </is>
       </c>
       <c r="O18" s="14" t="inlineStr">
@@ -11173,7 +11093,7 @@
       </c>
       <c r="P18" s="18" t="inlineStr">
         <is>
-          <t>@p0</t>
+          <t>@p1</t>
         </is>
       </c>
       <c r="Q18" s="22" t="inlineStr">
@@ -11193,24 +11113,19 @@
       </c>
       <c r="T18" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the workbook Upgrade &amp; Merge accept-all flow or company version generation.</t>
-        </is>
-      </c>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the workbook role-comparison screen needed for this color-coding validation.</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>failed: Current live Manage Company page does not expose the workbook Upgrade &amp; Merge accept-all f</t>
+          <t>failed: Current live Manage Company page does not expose the workbook role-comparison screen neede</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-018</t>
+          <t>COMP-E2E-012</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
@@ -11220,62 +11135,62 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Review individually</t>
+          <t>Add internal company role</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Verify Review Individually allows accepting some changes and keeping current for others</t>
+          <t>Verify company can add a new internal role</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Upgrade diff screen open</t>
+          <t>Company Admin logged in</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Mixed changes in upgrade diff</t>
+          <t>Unique internal role name</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>1. Open Review Individually 2. Accept one change 3. Keep Current for another 4. Save</t>
+          <t>1. Open Company Role Adjustments 2. Add new internal role 3. Save</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>System applies only accepted changes and preserves current values for kept items</t>
+          <t>New internal company role is added to the company variant</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>Functional / Versioning</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="K19" s="8" t="inlineStr">
         <is>
-          <t>Each change has [Accept] [Keep Current]</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L19" s="8" t="inlineStr">
         <is>
-          <t>Upgrade &amp; Merge Flow</t>
+          <t>Company role adjustments</t>
         </is>
       </c>
       <c r="M19" s="9" t="inlineStr">
         <is>
-          <t>Selective merge of company overrides</t>
+          <t>Add internal role</t>
         </is>
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>Industry version delta + company overrides</t>
+          <t>Company Admin logged in</t>
         </is>
       </c>
       <c r="O19" s="14" t="inlineStr">
@@ -11285,7 +11200,7 @@
       </c>
       <c r="P19" s="18" t="inlineStr">
         <is>
-          <t>@p0</t>
+          <t>@p1</t>
         </is>
       </c>
       <c r="Q19" s="22" t="inlineStr">
@@ -11305,24 +11220,19 @@
       </c>
       <c r="T19" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the workbook selective upgrade-merge decision flow.</t>
-        </is>
-      </c>
-      <c r="V19" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the company role-variant creation surface described in the workbook.</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>failed: Current live Manage Company page does not expose the workbook selective upgrade-merge deci</t>
+          <t>failed: Current live Manage Company page does not expose the company role-variant creation surface</t>
         </is>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>COMP-E2E-019</t>
+          <t>COMP-E2E-013</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
@@ -11332,37 +11242,37 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Defer upgrade</t>
+          <t>Adjust capability weight</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Verify company can defer an upgrade without changing the current company version</t>
+          <t>Verify company can adjust capability weights in the company role variant</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>Upgrade available state exists</t>
+          <t>Company role variant exists</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Company on old version with newer source version available</t>
+          <t>Changed weight for one mapped CI</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>1. Open upgrade flow 2. Click Defer Upgrade</t>
+          <t>1. Open a company role variant 2. Adjust capability weight 3. Save</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>Current company version remains unchanged and upgrade remains pending/available</t>
+          <t>Updated capability weight is saved in the company role variant</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>Functional / Versioning</t>
+          <t>Functional</t>
         </is>
       </c>
       <c r="J20" s="8" t="inlineStr">
@@ -11372,22 +11282,22 @@
       </c>
       <c r="K20" s="8" t="inlineStr">
         <is>
-          <t>Company option includes Defer Upgrade</t>
+          <t>Companies workbook</t>
         </is>
       </c>
       <c r="L20" s="8" t="inlineStr">
         <is>
-          <t>Upgrade &amp; Merge Flow</t>
+          <t>Company role adjustments</t>
         </is>
       </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>No version change on defer</t>
+          <t>Capability weight change</t>
         </is>
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
-          <t>Industry version delta + company version</t>
+          <t>Company role variant exists</t>
         </is>
       </c>
       <c r="O20" s="14" t="inlineStr">
@@ -11417,61 +11327,1404 @@
       </c>
       <c r="T20" s="13" t="inlineStr">
         <is>
-          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the workbook Defer Upgrade flow or company-WRCF version state.</t>
-        </is>
-      </c>
-      <c r="V20" t="inlineStr">
-        <is>
-          <t>not run</t>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose company role-variant capability weight adjustment.</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>failed: Current live Manage Company page does not expose the workbook Defer Upgrade flow or compan</t>
+          <t>failed: Current live Manage Company page does not expose company role-variant capability weight ad</t>
         </is>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="8" t="n"/>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
-      <c r="G21" s="8" t="n"/>
-      <c r="H21" s="8" t="n"/>
-      <c r="I21" s="8" t="n"/>
-      <c r="J21" s="8" t="n"/>
-      <c r="K21" s="8" t="n"/>
-      <c r="L21" s="8" t="n"/>
-      <c r="M21" s="9" t="n"/>
-      <c r="N21" s="8" t="n"/>
-      <c r="R21" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>COMP-E2E-014</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Companies</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Change certification threshold</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Verify company can change certification threshold in the company role variant</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Company role variant exists</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>New threshold value</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>1. Open company role variant 2. Change certification threshold 3. Save</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>Updated certification threshold is saved in the company role variant</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>Companies workbook</t>
+        </is>
+      </c>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>Company role adjustments</t>
+        </is>
+      </c>
+      <c r="M21" s="9" t="inlineStr">
+        <is>
+          <t>Certification threshold change</t>
+        </is>
+      </c>
+      <c r="N21" s="8" t="inlineStr">
+        <is>
+          <t>Company role variant exists</t>
+        </is>
+      </c>
+      <c r="O21" s="14" t="inlineStr">
+        <is>
+          <t>@future</t>
+        </is>
+      </c>
+      <c r="P21" s="18" t="inlineStr">
+        <is>
+          <t>@p1</t>
+        </is>
+      </c>
+      <c r="Q21" s="22" t="inlineStr">
+        <is>
+          <t>@companies</t>
+        </is>
+      </c>
+      <c r="R21" s="11" t="inlineStr">
         <is>
           <t>fail</t>
+        </is>
+      </c>
+      <c r="S21" s="11" t="inlineStr">
+        <is>
+          <t>product-gap</t>
+        </is>
+      </c>
+      <c r="T21" s="13" t="inlineStr">
+        <is>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose company role-variant certification-threshold override editing.</t>
+        </is>
+      </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>failed: Current live Manage Company page does not expose company role-variant certification-thresh</t>
         </is>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="8" t="n"/>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="8" t="n"/>
-      <c r="E22" s="8" t="n"/>
-      <c r="F22" s="8" t="n"/>
-      <c r="G22" s="8" t="n"/>
-      <c r="H22" s="8" t="n"/>
-      <c r="I22" s="8" t="n"/>
-      <c r="J22" s="8" t="n"/>
-      <c r="K22" s="8" t="n"/>
-      <c r="L22" s="8" t="n"/>
-      <c r="M22" s="9" t="n"/>
-      <c r="N22" s="8" t="n"/>
-      <c r="R22" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>COMP-E2E-015</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Companies</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade available indicator</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Verify company sees Upgrade Available when industry publishes a newer version</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Company references industry version 4.2; industry publishes 5.0</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>Newer published industry version available</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>1. Publish newer industry version 2. Open company dashboard</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>Dashboard shows Upgrade Available with the newer industry version</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>Functional / Versioning</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>Companies workbook</t>
+        </is>
+      </c>
+      <c r="L22" s="8" t="inlineStr">
+        <is>
+          <t>Company upgrade flow</t>
+        </is>
+      </c>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>Upgrade Available</t>
+        </is>
+      </c>
+      <c r="N22" s="8" t="inlineStr">
+        <is>
+          <t>Newer industry version</t>
+        </is>
+      </c>
+      <c r="O22" s="14" t="inlineStr">
+        <is>
+          <t>@future</t>
+        </is>
+      </c>
+      <c r="P22" s="18" t="inlineStr">
+        <is>
+          <t>@p0</t>
+        </is>
+      </c>
+      <c r="Q22" s="22" t="inlineStr">
+        <is>
+          <t>@companies</t>
+        </is>
+      </c>
+      <c r="R22" s="11" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
       </c>
+      <c r="S22" s="11" t="inlineStr">
+        <is>
+          <t>product-gap</t>
+        </is>
+      </c>
+      <c r="T22" s="13" t="inlineStr">
+        <is>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose industry/company WRCF version comparison or Upgrade Available state.</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">failed: Current live Manage Company page does not expose industry/company WRCF version comparison </t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>COMP-E2E-016</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Companies</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade diff screen</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Verify upgrade flow shows diffs before applying update</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade available state exists</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Changes include new CI / modified escalation / updated regulatory refs</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>1. Open Upgrade Available 2. Review diff screen</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>System shows differences such as new capability instances, modified escalation levels, and updated regulatory references</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Functional / Versioning</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>Companies workbook</t>
+        </is>
+      </c>
+      <c r="L23" s="8" t="inlineStr">
+        <is>
+          <t>Company upgrade flow</t>
+        </is>
+      </c>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>Upgrade diff screen</t>
+        </is>
+      </c>
+      <c r="N23" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade available state</t>
+        </is>
+      </c>
+      <c r="O23" s="14" t="inlineStr">
+        <is>
+          <t>@future</t>
+        </is>
+      </c>
+      <c r="P23" s="18" t="inlineStr">
+        <is>
+          <t>@p0</t>
+        </is>
+      </c>
+      <c r="Q23" s="22" t="inlineStr">
+        <is>
+          <t>@companies</t>
+        </is>
+      </c>
+      <c r="R23" s="11" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="S23" s="11" t="inlineStr">
+        <is>
+          <t>product-gap</t>
+        </is>
+      </c>
+      <c r="T23" s="13" t="inlineStr">
+        <is>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the workbook Upgrade &amp; Merge diff flow.</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>failed: Current live Manage Company page does not expose the workbook Upgrade &amp; Merge diff flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>COMP-E2E-017</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Companies</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Accept all upgrade</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Verify Accept All applies all industry updates and generates the next company version</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade available state exists</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Company on 4.2-C1; industry on 5.0</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>1. Open upgrade flow 2. Click Accept All 3. Confirm</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>All applicable updates are applied and a new company version is generated</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Functional / Versioning</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>Companies workbook</t>
+        </is>
+      </c>
+      <c r="L24" s="8" t="inlineStr">
+        <is>
+          <t>Company upgrade flow</t>
+        </is>
+      </c>
+      <c r="M24" s="9" t="inlineStr">
+        <is>
+          <t>Accept all upgrade</t>
+        </is>
+      </c>
+      <c r="N24" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade available state</t>
+        </is>
+      </c>
+      <c r="O24" s="14" t="inlineStr">
+        <is>
+          <t>@future</t>
+        </is>
+      </c>
+      <c r="P24" s="18" t="inlineStr">
+        <is>
+          <t>@p0</t>
+        </is>
+      </c>
+      <c r="Q24" s="22" t="inlineStr">
+        <is>
+          <t>@companies</t>
+        </is>
+      </c>
+      <c r="R24" s="11" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="S24" s="11" t="inlineStr">
+        <is>
+          <t>product-gap</t>
+        </is>
+      </c>
+      <c r="T24" s="13" t="inlineStr">
+        <is>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the workbook Upgrade &amp; Merge accept-all flow or company version generation.</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>failed: Current live Manage Company page does not expose the workbook Upgrade &amp; Merge accept-all f</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>COMP-E2E-018</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Companies</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Review individually</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Verify Review Individually allows accepting some changes and keeping current for others</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade diff screen open</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Mixed changes in upgrade diff</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>1. Open Review Individually 2. Accept one change 3. Keep Current for another 4. Save</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>System applies only accepted changes and preserves current values for kept items</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>Functional / Versioning</t>
+        </is>
+      </c>
+      <c r="J25" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>Companies workbook</t>
+        </is>
+      </c>
+      <c r="L25" s="8" t="inlineStr">
+        <is>
+          <t>Company upgrade flow</t>
+        </is>
+      </c>
+      <c r="M25" s="9" t="inlineStr">
+        <is>
+          <t>Review individually</t>
+        </is>
+      </c>
+      <c r="N25" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade diff screen open</t>
+        </is>
+      </c>
+      <c r="O25" s="14" t="inlineStr">
+        <is>
+          <t>@future</t>
+        </is>
+      </c>
+      <c r="P25" s="18" t="inlineStr">
+        <is>
+          <t>@p0</t>
+        </is>
+      </c>
+      <c r="Q25" s="22" t="inlineStr">
+        <is>
+          <t>@companies</t>
+        </is>
+      </c>
+      <c r="R25" s="11" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="S25" s="11" t="inlineStr">
+        <is>
+          <t>product-gap</t>
+        </is>
+      </c>
+      <c r="T25" s="13" t="inlineStr">
+        <is>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the workbook selective upgrade-merge decision flow.</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>failed: Current live Manage Company page does not expose the workbook selective upgrade-merge deci</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>COMP-E2E-019</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Companies</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Defer upgrade</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Verify company can defer an upgrade without changing the current company version</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade available state exists</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>Company on old version with newer source version available</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>1. Open upgrade flow 2. Click Defer Upgrade</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>Current company version remains unchanged and upgrade remains pending/available</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>Functional / Versioning</t>
+        </is>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K26" s="8" t="inlineStr">
+        <is>
+          <t>Companies workbook</t>
+        </is>
+      </c>
+      <c r="L26" s="8" t="inlineStr">
+        <is>
+          <t>Company upgrade flow</t>
+        </is>
+      </c>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>Defer upgrade</t>
+        </is>
+      </c>
+      <c r="N26" s="8" t="inlineStr">
+        <is>
+          <t>Upgrade available state</t>
+        </is>
+      </c>
+      <c r="O26" s="14" t="inlineStr">
+        <is>
+          <t>@future</t>
+        </is>
+      </c>
+      <c r="P26" s="18" t="inlineStr">
+        <is>
+          <t>@p1</t>
+        </is>
+      </c>
+      <c r="Q26" s="22" t="inlineStr">
+        <is>
+          <t>@companies</t>
+        </is>
+      </c>
+      <c r="R26" s="11" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="S26" s="11" t="inlineStr">
+        <is>
+          <t>product-gap</t>
+        </is>
+      </c>
+      <c r="T26" s="13" t="inlineStr">
+        <is>
+          <t>Failed in the 11:11 PM @ 03/04/26 rerun: Current live Manage Company page does not expose the workbook Defer Upgrade flow or company-WRCF version state.</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>failed: Current live Manage Company page does not expose the workbook Defer Upgrade flow or compan</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="8" t="n"/>
+      <c r="H27" s="8" t="n"/>
+      <c r="I27" s="8" t="n"/>
+      <c r="J27" s="8" t="n"/>
+      <c r="K27" s="8" t="n"/>
+      <c r="L27" s="8" t="n"/>
+      <c r="M27" s="9" t="n"/>
+      <c r="N27" s="8" t="n"/>
+      <c r="O27" s="14" t="n"/>
+      <c r="P27" s="18" t="n"/>
+      <c r="Q27" s="22" t="n"/>
+      <c r="R27" s="11" t="n"/>
+      <c r="S27" s="11" t="n"/>
+      <c r="T27" s="13" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="8" t="n"/>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="8" t="n"/>
+      <c r="H28" s="8" t="n"/>
+      <c r="I28" s="8" t="n"/>
+      <c r="J28" s="8" t="n"/>
+      <c r="K28" s="8" t="n"/>
+      <c r="L28" s="8" t="n"/>
+      <c r="M28" s="9" t="n"/>
+      <c r="N28" s="8" t="n"/>
+      <c r="O28" s="14" t="n"/>
+      <c r="P28" s="18" t="n"/>
+      <c r="Q28" s="22" t="n"/>
+      <c r="R28" s="11" t="n"/>
+      <c r="S28" s="11" t="n"/>
+      <c r="T28" s="13" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="8" t="n"/>
+      <c r="G29" s="8" t="n"/>
+      <c r="H29" s="8" t="n"/>
+      <c r="I29" s="8" t="n"/>
+      <c r="J29" s="8" t="n"/>
+      <c r="K29" s="8" t="n"/>
+      <c r="L29" s="8" t="n"/>
+      <c r="M29" s="9" t="n"/>
+      <c r="N29" s="8" t="n"/>
+      <c r="O29" s="14" t="n"/>
+      <c r="P29" s="18" t="n"/>
+      <c r="Q29" s="22" t="n"/>
+      <c r="R29" s="11" t="n"/>
+      <c r="S29" s="11" t="n"/>
+      <c r="T29" s="13" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="8" t="n"/>
+      <c r="H30" s="8" t="n"/>
+      <c r="I30" s="8" t="n"/>
+      <c r="J30" s="8" t="n"/>
+      <c r="K30" s="8" t="n"/>
+      <c r="L30" s="8" t="n"/>
+      <c r="M30" s="9" t="n"/>
+      <c r="N30" s="8" t="n"/>
+      <c r="O30" s="14" t="n"/>
+      <c r="P30" s="18" t="n"/>
+      <c r="Q30" s="22" t="n"/>
+      <c r="R30" s="11" t="n"/>
+      <c r="S30" s="11" t="n"/>
+      <c r="T30" s="13" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="8" t="n"/>
+      <c r="H31" s="8" t="n"/>
+      <c r="I31" s="8" t="n"/>
+      <c r="J31" s="8" t="n"/>
+      <c r="K31" s="8" t="n"/>
+      <c r="L31" s="8" t="n"/>
+      <c r="M31" s="9" t="n"/>
+      <c r="N31" s="8" t="n"/>
+      <c r="O31" s="14" t="n"/>
+      <c r="P31" s="18" t="n"/>
+      <c r="Q31" s="22" t="n"/>
+      <c r="R31" s="11" t="n"/>
+      <c r="S31" s="11" t="n"/>
+      <c r="T31" s="13" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="8" t="n"/>
+      <c r="H32" s="8" t="n"/>
+      <c r="I32" s="8" t="n"/>
+      <c r="J32" s="8" t="n"/>
+      <c r="K32" s="8" t="n"/>
+      <c r="L32" s="8" t="n"/>
+      <c r="M32" s="9" t="n"/>
+      <c r="N32" s="8" t="n"/>
+      <c r="O32" s="14" t="n"/>
+      <c r="P32" s="18" t="n"/>
+      <c r="Q32" s="22" t="n"/>
+      <c r="R32" s="11" t="n"/>
+      <c r="S32" s="11" t="n"/>
+      <c r="T32" s="13" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="8" t="n"/>
+      <c r="H33" s="8" t="n"/>
+      <c r="I33" s="8" t="n"/>
+      <c r="J33" s="8" t="n"/>
+      <c r="K33" s="8" t="n"/>
+      <c r="L33" s="8" t="n"/>
+      <c r="M33" s="9" t="n"/>
+      <c r="N33" s="8" t="n"/>
+      <c r="O33" s="14" t="n"/>
+      <c r="P33" s="18" t="n"/>
+      <c r="Q33" s="22" t="n"/>
+      <c r="R33" s="11" t="n"/>
+      <c r="S33" s="11" t="n"/>
+      <c r="T33" s="13" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="8" t="n"/>
+      <c r="E34" s="8" t="n"/>
+      <c r="F34" s="8" t="n"/>
+      <c r="G34" s="8" t="n"/>
+      <c r="H34" s="8" t="n"/>
+      <c r="I34" s="8" t="n"/>
+      <c r="J34" s="8" t="n"/>
+      <c r="K34" s="8" t="n"/>
+      <c r="L34" s="8" t="n"/>
+      <c r="M34" s="9" t="n"/>
+      <c r="N34" s="8" t="n"/>
+      <c r="O34" s="14" t="n"/>
+      <c r="P34" s="18" t="n"/>
+      <c r="Q34" s="22" t="n"/>
+      <c r="R34" s="11" t="n"/>
+      <c r="S34" s="11" t="n"/>
+      <c r="T34" s="13" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n"/>
+      <c r="B35" s="8" t="n"/>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="8" t="n"/>
+      <c r="E35" s="8" t="n"/>
+      <c r="F35" s="8" t="n"/>
+      <c r="G35" s="8" t="n"/>
+      <c r="H35" s="8" t="n"/>
+      <c r="I35" s="8" t="n"/>
+      <c r="J35" s="8" t="n"/>
+      <c r="K35" s="8" t="n"/>
+      <c r="L35" s="8" t="n"/>
+      <c r="M35" s="9" t="n"/>
+      <c r="N35" s="8" t="n"/>
+      <c r="O35" s="14" t="n"/>
+      <c r="P35" s="18" t="n"/>
+      <c r="Q35" s="22" t="n"/>
+      <c r="R35" s="11" t="n"/>
+      <c r="S35" s="11" t="n"/>
+      <c r="T35" s="13" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n"/>
+      <c r="B36" s="8" t="n"/>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="8" t="n"/>
+      <c r="E36" s="8" t="n"/>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="8" t="n"/>
+      <c r="H36" s="8" t="n"/>
+      <c r="I36" s="8" t="n"/>
+      <c r="J36" s="8" t="n"/>
+      <c r="K36" s="8" t="n"/>
+      <c r="L36" s="8" t="n"/>
+      <c r="M36" s="9" t="n"/>
+      <c r="N36" s="8" t="n"/>
+      <c r="O36" s="14" t="n"/>
+      <c r="P36" s="18" t="n"/>
+      <c r="Q36" s="22" t="n"/>
+      <c r="R36" s="11" t="n"/>
+      <c r="S36" s="11" t="n"/>
+      <c r="T36" s="13" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="8" t="n"/>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="8" t="n"/>
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="8" t="n"/>
+      <c r="H37" s="8" t="n"/>
+      <c r="I37" s="8" t="n"/>
+      <c r="J37" s="8" t="n"/>
+      <c r="K37" s="8" t="n"/>
+      <c r="L37" s="8" t="n"/>
+      <c r="M37" s="9" t="n"/>
+      <c r="N37" s="8" t="n"/>
+      <c r="O37" s="14" t="n"/>
+      <c r="P37" s="18" t="n"/>
+      <c r="Q37" s="22" t="n"/>
+      <c r="R37" s="11" t="n"/>
+      <c r="S37" s="11" t="n"/>
+      <c r="T37" s="13" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n"/>
+      <c r="B38" s="8" t="n"/>
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="8" t="n"/>
+      <c r="E38" s="8" t="n"/>
+      <c r="F38" s="8" t="n"/>
+      <c r="G38" s="8" t="n"/>
+      <c r="H38" s="8" t="n"/>
+      <c r="I38" s="8" t="n"/>
+      <c r="J38" s="8" t="n"/>
+      <c r="K38" s="8" t="n"/>
+      <c r="L38" s="8" t="n"/>
+      <c r="M38" s="9" t="n"/>
+      <c r="N38" s="8" t="n"/>
+      <c r="O38" s="14" t="n"/>
+      <c r="P38" s="18" t="n"/>
+      <c r="Q38" s="22" t="n"/>
+      <c r="R38" s="11" t="n"/>
+      <c r="S38" s="11" t="n"/>
+      <c r="T38" s="13" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n"/>
+      <c r="B39" s="8" t="n"/>
+      <c r="C39" s="8" t="n"/>
+      <c r="D39" s="8" t="n"/>
+      <c r="E39" s="8" t="n"/>
+      <c r="F39" s="8" t="n"/>
+      <c r="G39" s="8" t="n"/>
+      <c r="H39" s="8" t="n"/>
+      <c r="I39" s="8" t="n"/>
+      <c r="J39" s="8" t="n"/>
+      <c r="K39" s="8" t="n"/>
+      <c r="L39" s="8" t="n"/>
+      <c r="M39" s="9" t="n"/>
+      <c r="N39" s="8" t="n"/>
+      <c r="O39" s="14" t="n"/>
+      <c r="P39" s="18" t="n"/>
+      <c r="Q39" s="22" t="n"/>
+      <c r="R39" s="11" t="n"/>
+      <c r="S39" s="11" t="n"/>
+      <c r="T39" s="13" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n"/>
+      <c r="B40" s="8" t="n"/>
+      <c r="C40" s="8" t="n"/>
+      <c r="D40" s="8" t="n"/>
+      <c r="E40" s="8" t="n"/>
+      <c r="F40" s="8" t="n"/>
+      <c r="G40" s="8" t="n"/>
+      <c r="H40" s="8" t="n"/>
+      <c r="I40" s="8" t="n"/>
+      <c r="J40" s="8" t="n"/>
+      <c r="K40" s="8" t="n"/>
+      <c r="L40" s="8" t="n"/>
+      <c r="M40" s="9" t="n"/>
+      <c r="N40" s="8" t="n"/>
+      <c r="O40" s="14" t="n"/>
+      <c r="P40" s="18" t="n"/>
+      <c r="Q40" s="22" t="n"/>
+      <c r="R40" s="11" t="n"/>
+      <c r="S40" s="11" t="n"/>
+      <c r="T40" s="13" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n"/>
+      <c r="B41" s="8" t="n"/>
+      <c r="C41" s="8" t="n"/>
+      <c r="D41" s="8" t="n"/>
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="8" t="n"/>
+      <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
+      <c r="J41" s="8" t="n"/>
+      <c r="K41" s="8" t="n"/>
+      <c r="L41" s="8" t="n"/>
+      <c r="M41" s="9" t="n"/>
+      <c r="N41" s="8" t="n"/>
+      <c r="O41" s="14" t="n"/>
+      <c r="P41" s="18" t="n"/>
+      <c r="Q41" s="22" t="n"/>
+      <c r="R41" s="11" t="n"/>
+      <c r="S41" s="11" t="n"/>
+      <c r="T41" s="13" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
+      <c r="H42" s="8" t="n"/>
+      <c r="I42" s="8" t="n"/>
+      <c r="J42" s="8" t="n"/>
+      <c r="K42" s="8" t="n"/>
+      <c r="L42" s="8" t="n"/>
+      <c r="M42" s="9" t="n"/>
+      <c r="N42" s="8" t="n"/>
+      <c r="O42" s="14" t="n"/>
+      <c r="P42" s="18" t="n"/>
+      <c r="Q42" s="22" t="n"/>
+      <c r="R42" s="11" t="n"/>
+      <c r="S42" s="11" t="n"/>
+      <c r="T42" s="13" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n"/>
+      <c r="B43" s="8" t="n"/>
+      <c r="C43" s="8" t="n"/>
+      <c r="D43" s="8" t="n"/>
+      <c r="E43" s="8" t="n"/>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="8" t="n"/>
+      <c r="H43" s="8" t="n"/>
+      <c r="I43" s="8" t="n"/>
+      <c r="J43" s="8" t="n"/>
+      <c r="K43" s="8" t="n"/>
+      <c r="L43" s="8" t="n"/>
+      <c r="M43" s="9" t="n"/>
+      <c r="N43" s="8" t="n"/>
+      <c r="O43" s="14" t="n"/>
+      <c r="P43" s="18" t="n"/>
+      <c r="Q43" s="22" t="n"/>
+      <c r="R43" s="11" t="n"/>
+      <c r="S43" s="11" t="n"/>
+      <c r="T43" s="13" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n"/>
+      <c r="B44" s="8" t="n"/>
+      <c r="C44" s="8" t="n"/>
+      <c r="D44" s="8" t="n"/>
+      <c r="E44" s="8" t="n"/>
+      <c r="F44" s="8" t="n"/>
+      <c r="G44" s="8" t="n"/>
+      <c r="H44" s="8" t="n"/>
+      <c r="I44" s="8" t="n"/>
+      <c r="J44" s="8" t="n"/>
+      <c r="K44" s="8" t="n"/>
+      <c r="L44" s="8" t="n"/>
+      <c r="M44" s="9" t="n"/>
+      <c r="N44" s="8" t="n"/>
+      <c r="O44" s="14" t="n"/>
+      <c r="P44" s="18" t="n"/>
+      <c r="Q44" s="22" t="n"/>
+      <c r="R44" s="11" t="n"/>
+      <c r="S44" s="11" t="n"/>
+      <c r="T44" s="13" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n"/>
+      <c r="B45" s="8" t="n"/>
+      <c r="C45" s="8" t="n"/>
+      <c r="D45" s="8" t="n"/>
+      <c r="E45" s="8" t="n"/>
+      <c r="F45" s="8" t="n"/>
+      <c r="G45" s="8" t="n"/>
+      <c r="H45" s="8" t="n"/>
+      <c r="I45" s="8" t="n"/>
+      <c r="J45" s="8" t="n"/>
+      <c r="K45" s="8" t="n"/>
+      <c r="L45" s="8" t="n"/>
+      <c r="M45" s="9" t="n"/>
+      <c r="N45" s="8" t="n"/>
+      <c r="O45" s="14" t="n"/>
+      <c r="P45" s="18" t="n"/>
+      <c r="Q45" s="22" t="n"/>
+      <c r="R45" s="11" t="n"/>
+      <c r="S45" s="11" t="n"/>
+      <c r="T45" s="13" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n"/>
+      <c r="B46" s="8" t="n"/>
+      <c r="C46" s="8" t="n"/>
+      <c r="D46" s="8" t="n"/>
+      <c r="E46" s="8" t="n"/>
+      <c r="F46" s="8" t="n"/>
+      <c r="G46" s="8" t="n"/>
+      <c r="H46" s="8" t="n"/>
+      <c r="I46" s="8" t="n"/>
+      <c r="J46" s="8" t="n"/>
+      <c r="K46" s="8" t="n"/>
+      <c r="L46" s="8" t="n"/>
+      <c r="M46" s="9" t="n"/>
+      <c r="N46" s="8" t="n"/>
+      <c r="O46" s="14" t="n"/>
+      <c r="P46" s="18" t="n"/>
+      <c r="Q46" s="22" t="n"/>
+      <c r="R46" s="11" t="n"/>
+      <c r="S46" s="11" t="n"/>
+      <c r="T46" s="13" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="n"/>
+      <c r="B47" s="8" t="n"/>
+      <c r="C47" s="8" t="n"/>
+      <c r="D47" s="8" t="n"/>
+      <c r="E47" s="8" t="n"/>
+      <c r="F47" s="8" t="n"/>
+      <c r="G47" s="8" t="n"/>
+      <c r="H47" s="8" t="n"/>
+      <c r="I47" s="8" t="n"/>
+      <c r="J47" s="8" t="n"/>
+      <c r="K47" s="8" t="n"/>
+      <c r="L47" s="8" t="n"/>
+      <c r="M47" s="9" t="n"/>
+      <c r="N47" s="8" t="n"/>
+      <c r="O47" s="14" t="n"/>
+      <c r="P47" s="18" t="n"/>
+      <c r="Q47" s="22" t="n"/>
+      <c r="R47" s="11" t="n"/>
+      <c r="S47" s="11" t="n"/>
+      <c r="T47" s="13" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n"/>
+      <c r="B48" s="8" t="n"/>
+      <c r="C48" s="8" t="n"/>
+      <c r="D48" s="8" t="n"/>
+      <c r="E48" s="8" t="n"/>
+      <c r="F48" s="8" t="n"/>
+      <c r="G48" s="8" t="n"/>
+      <c r="H48" s="8" t="n"/>
+      <c r="I48" s="8" t="n"/>
+      <c r="J48" s="8" t="n"/>
+      <c r="K48" s="8" t="n"/>
+      <c r="L48" s="8" t="n"/>
+      <c r="M48" s="9" t="n"/>
+      <c r="N48" s="8" t="n"/>
+      <c r="O48" s="14" t="n"/>
+      <c r="P48" s="18" t="n"/>
+      <c r="Q48" s="22" t="n"/>
+      <c r="R48" s="11" t="n"/>
+      <c r="S48" s="11" t="n"/>
+      <c r="T48" s="13" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="8" t="n"/>
+      <c r="C49" s="8" t="n"/>
+      <c r="D49" s="8" t="n"/>
+      <c r="E49" s="8" t="n"/>
+      <c r="F49" s="8" t="n"/>
+      <c r="G49" s="8" t="n"/>
+      <c r="H49" s="8" t="n"/>
+      <c r="I49" s="8" t="n"/>
+      <c r="J49" s="8" t="n"/>
+      <c r="K49" s="8" t="n"/>
+      <c r="L49" s="8" t="n"/>
+      <c r="M49" s="9" t="n"/>
+      <c r="N49" s="8" t="n"/>
+      <c r="O49" s="14" t="n"/>
+      <c r="P49" s="18" t="n"/>
+      <c r="Q49" s="22" t="n"/>
+      <c r="R49" s="11" t="n"/>
+      <c r="S49" s="11" t="n"/>
+      <c r="T49" s="13" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n"/>
+      <c r="B50" s="8" t="n"/>
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="8" t="n"/>
+      <c r="E50" s="8" t="n"/>
+      <c r="F50" s="8" t="n"/>
+      <c r="G50" s="8" t="n"/>
+      <c r="H50" s="8" t="n"/>
+      <c r="I50" s="8" t="n"/>
+      <c r="J50" s="8" t="n"/>
+      <c r="K50" s="8" t="n"/>
+      <c r="L50" s="8" t="n"/>
+      <c r="M50" s="9" t="n"/>
+      <c r="N50" s="8" t="n"/>
+      <c r="O50" s="14" t="n"/>
+      <c r="P50" s="18" t="n"/>
+      <c r="Q50" s="22" t="n"/>
+      <c r="R50" s="11" t="n"/>
+      <c r="S50" s="11" t="n"/>
+      <c r="T50" s="13" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n"/>
+      <c r="B51" s="8" t="n"/>
+      <c r="C51" s="8" t="n"/>
+      <c r="D51" s="8" t="n"/>
+      <c r="E51" s="8" t="n"/>
+      <c r="F51" s="8" t="n"/>
+      <c r="G51" s="8" t="n"/>
+      <c r="H51" s="8" t="n"/>
+      <c r="I51" s="8" t="n"/>
+      <c r="J51" s="8" t="n"/>
+      <c r="K51" s="8" t="n"/>
+      <c r="L51" s="8" t="n"/>
+      <c r="M51" s="9" t="n"/>
+      <c r="N51" s="8" t="n"/>
+      <c r="O51" s="14" t="n"/>
+      <c r="P51" s="18" t="n"/>
+      <c r="Q51" s="22" t="n"/>
+      <c r="R51" s="11" t="n"/>
+      <c r="S51" s="11" t="n"/>
+      <c r="T51" s="13" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n"/>
+      <c r="B52" s="8" t="n"/>
+      <c r="C52" s="8" t="n"/>
+      <c r="D52" s="8" t="n"/>
+      <c r="E52" s="8" t="n"/>
+      <c r="F52" s="8" t="n"/>
+      <c r="G52" s="8" t="n"/>
+      <c r="H52" s="8" t="n"/>
+      <c r="I52" s="8" t="n"/>
+      <c r="J52" s="8" t="n"/>
+      <c r="K52" s="8" t="n"/>
+      <c r="L52" s="8" t="n"/>
+      <c r="M52" s="9" t="n"/>
+      <c r="N52" s="8" t="n"/>
+      <c r="O52" s="14" t="n"/>
+      <c r="P52" s="18" t="n"/>
+      <c r="Q52" s="22" t="n"/>
+      <c r="R52" s="11" t="n"/>
+      <c r="S52" s="11" t="n"/>
+      <c r="T52" s="13" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="n"/>
+      <c r="B53" s="8" t="n"/>
+      <c r="C53" s="8" t="n"/>
+      <c r="D53" s="8" t="n"/>
+      <c r="E53" s="8" t="n"/>
+      <c r="F53" s="8" t="n"/>
+      <c r="G53" s="8" t="n"/>
+      <c r="H53" s="8" t="n"/>
+      <c r="I53" s="8" t="n"/>
+      <c r="J53" s="8" t="n"/>
+      <c r="K53" s="8" t="n"/>
+      <c r="L53" s="8" t="n"/>
+      <c r="M53" s="9" t="n"/>
+      <c r="N53" s="8" t="n"/>
+      <c r="O53" s="14" t="n"/>
+      <c r="P53" s="18" t="n"/>
+      <c r="Q53" s="22" t="n"/>
+      <c r="R53" s="11" t="n"/>
+      <c r="S53" s="11" t="n"/>
+      <c r="T53" s="13" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n"/>
+      <c r="B54" s="8" t="n"/>
+      <c r="C54" s="8" t="n"/>
+      <c r="D54" s="8" t="n"/>
+      <c r="E54" s="8" t="n"/>
+      <c r="F54" s="8" t="n"/>
+      <c r="G54" s="8" t="n"/>
+      <c r="H54" s="8" t="n"/>
+      <c r="I54" s="8" t="n"/>
+      <c r="J54" s="8" t="n"/>
+      <c r="K54" s="8" t="n"/>
+      <c r="L54" s="8" t="n"/>
+      <c r="M54" s="9" t="n"/>
+      <c r="N54" s="8" t="n"/>
+      <c r="O54" s="14" t="n"/>
+      <c r="P54" s="18" t="n"/>
+      <c r="Q54" s="22" t="n"/>
+      <c r="R54" s="11" t="n"/>
+      <c r="S54" s="11" t="n"/>
+      <c r="T54" s="13" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="n"/>
+      <c r="B55" s="8" t="n"/>
+      <c r="C55" s="8" t="n"/>
+      <c r="D55" s="8" t="n"/>
+      <c r="E55" s="8" t="n"/>
+      <c r="F55" s="8" t="n"/>
+      <c r="G55" s="8" t="n"/>
+      <c r="H55" s="8" t="n"/>
+      <c r="I55" s="8" t="n"/>
+      <c r="J55" s="8" t="n"/>
+      <c r="K55" s="8" t="n"/>
+      <c r="L55" s="8" t="n"/>
+      <c r="M55" s="9" t="n"/>
+      <c r="N55" s="8" t="n"/>
+      <c r="O55" s="14" t="n"/>
+      <c r="P55" s="18" t="n"/>
+      <c r="Q55" s="22" t="n"/>
+      <c r="R55" s="11" t="n"/>
+      <c r="S55" s="11" t="n"/>
+      <c r="T55" s="13" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n"/>
+      <c r="B56" s="8" t="n"/>
+      <c r="C56" s="8" t="n"/>
+      <c r="D56" s="8" t="n"/>
+      <c r="E56" s="8" t="n"/>
+      <c r="F56" s="8" t="n"/>
+      <c r="G56" s="8" t="n"/>
+      <c r="H56" s="8" t="n"/>
+      <c r="I56" s="8" t="n"/>
+      <c r="J56" s="8" t="n"/>
+      <c r="K56" s="8" t="n"/>
+      <c r="L56" s="8" t="n"/>
+      <c r="M56" s="9" t="n"/>
+      <c r="N56" s="8" t="n"/>
+      <c r="O56" s="14" t="n"/>
+      <c r="P56" s="18" t="n"/>
+      <c r="Q56" s="22" t="n"/>
+      <c r="R56" s="11" t="n"/>
+      <c r="S56" s="11" t="n"/>
+      <c r="T56" s="13" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="n"/>
+      <c r="B57" s="8" t="n"/>
+      <c r="C57" s="8" t="n"/>
+      <c r="D57" s="8" t="n"/>
+      <c r="E57" s="8" t="n"/>
+      <c r="F57" s="8" t="n"/>
+      <c r="G57" s="8" t="n"/>
+      <c r="H57" s="8" t="n"/>
+      <c r="I57" s="8" t="n"/>
+      <c r="J57" s="8" t="n"/>
+      <c r="K57" s="8" t="n"/>
+      <c r="L57" s="8" t="n"/>
+      <c r="M57" s="9" t="n"/>
+      <c r="N57" s="8" t="n"/>
+      <c r="O57" s="14" t="n"/>
+      <c r="P57" s="18" t="n"/>
+      <c r="Q57" s="22" t="n"/>
+      <c r="R57" s="11" t="n"/>
+      <c r="S57" s="11" t="n"/>
+      <c r="T57" s="13" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n"/>
+      <c r="B58" s="8" t="n"/>
+      <c r="C58" s="8" t="n"/>
+      <c r="D58" s="8" t="n"/>
+      <c r="E58" s="8" t="n"/>
+      <c r="F58" s="8" t="n"/>
+      <c r="G58" s="8" t="n"/>
+      <c r="H58" s="8" t="n"/>
+      <c r="I58" s="8" t="n"/>
+      <c r="J58" s="8" t="n"/>
+      <c r="K58" s="8" t="n"/>
+      <c r="L58" s="8" t="n"/>
+      <c r="M58" s="9" t="n"/>
+      <c r="N58" s="8" t="n"/>
+      <c r="O58" s="14" t="n"/>
+      <c r="P58" s="18" t="n"/>
+      <c r="Q58" s="22" t="n"/>
+      <c r="R58" s="11" t="n"/>
+      <c r="S58" s="11" t="n"/>
+      <c r="T58" s="13" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="n"/>
+      <c r="B59" s="8" t="n"/>
+      <c r="C59" s="8" t="n"/>
+      <c r="D59" s="8" t="n"/>
+      <c r="E59" s="8" t="n"/>
+      <c r="F59" s="8" t="n"/>
+      <c r="G59" s="8" t="n"/>
+      <c r="H59" s="8" t="n"/>
+      <c r="I59" s="8" t="n"/>
+      <c r="J59" s="8" t="n"/>
+      <c r="K59" s="8" t="n"/>
+      <c r="L59" s="8" t="n"/>
+      <c r="M59" s="9" t="n"/>
+      <c r="N59" s="8" t="n"/>
+      <c r="O59" s="14" t="n"/>
+      <c r="P59" s="18" t="n"/>
+      <c r="Q59" s="22" t="n"/>
+      <c r="R59" s="11" t="n"/>
+      <c r="S59" s="11" t="n"/>
+      <c r="T59" s="13" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="n"/>
+      <c r="B60" s="8" t="n"/>
+      <c r="C60" s="8" t="n"/>
+      <c r="D60" s="8" t="n"/>
+      <c r="E60" s="8" t="n"/>
+      <c r="F60" s="8" t="n"/>
+      <c r="G60" s="8" t="n"/>
+      <c r="H60" s="8" t="n"/>
+      <c r="I60" s="8" t="n"/>
+      <c r="J60" s="8" t="n"/>
+      <c r="K60" s="8" t="n"/>
+      <c r="L60" s="8" t="n"/>
+      <c r="M60" s="9" t="n"/>
+      <c r="N60" s="8" t="n"/>
+      <c r="O60" s="14" t="n"/>
+      <c r="P60" s="18" t="n"/>
+      <c r="Q60" s="22" t="n"/>
+      <c r="R60" s="11" t="n"/>
+      <c r="S60" s="11" t="n"/>
+      <c r="T60" s="13" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>

</xml_diff>